<commit_message>
Add monthly subscription (Ad packages) developer brief + tasks
- docs/11-subscriptions-ad-packages.md: Stripe subscription brief for monthly
  Ad packages (e.g. 5 brand ad creatives + 3 ad videos/month). Generic
  multi-tier plan/quota model, use-it-or-lose-it reset on invoice.paid, block
  on exhaustion, cancel at period end via Stripe Customer Portal, webhooks,
  quota enforcement, UI; Tolt commission applies to subs too
- Add S1-S6 tasks to both Excel backlogs (EN dev + DE), link from docs/10 + README

https://claude.ai/code/session_013JDpec7ycgLb5kBriwRot4
</commit_message>
<xml_diff>
--- a/AMZVisuals_Developer_ToDo_EN.xlsx
+++ b/AMZVisuals_Developer_ToDo_EN.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Context &amp; Architecture" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Developer To-Do'!$A$3:$K$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Developer To-Do'!$A$3:$K$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2153,7 +2153,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>ARCH1</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
@@ -2163,32 +2163,32 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Architecture</t>
-        </is>
-      </c>
-      <c r="D35" s="15" t="inlineStr">
-        <is>
-          <t>Architecture</t>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>Multi-tenancy / org_id from day 1</t>
+          <t>Stripe subscription + Customer Portal</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>Introduce org_id / tenant_id in the data model, auth &amp; storage now (even if full white-label comes later). Retrofitting is expensive.</t>
+          <t>New monthly recurring plans parallel to one-time services (e.g. 'Ad Premium Package' = 5 brand ad creatives + 3 ad videos/month). Stripe Product + recurring monthly Price, Checkout in subscription mode. Enable Stripe Customer Portal for self-serve cancel (at period end), card update, invoices = near-zero dev.</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>handoff</t>
+          <t>decision 13.06</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr"/>
@@ -2202,42 +2202,42 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>ARCH2</t>
-        </is>
-      </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Architecture</t>
-        </is>
-      </c>
-      <c r="D36" s="15" t="inlineStr">
-        <is>
-          <t>Architecture</t>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>Async jobs / queue</t>
+          <t>Plan/quota data model (generic, multi-tier)</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Run AI generation &amp; video rendering via a queue + status + webhooks; never synchronously inside the request.</t>
+          <t>Data-driven plans with monthly quotas JSON e.g. {ad_creative:5, ad_video:3}; subscriptions + per-period quota_usage tables tied to org_id. Build GENERIC (multiple tiers planned), not hardcoded to one package.</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>handoff</t>
+          <t>decision 13.06</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr"/>
@@ -2251,42 +2251,42 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>ARCH3</t>
-        </is>
-      </c>
-      <c r="B37" s="14" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Architecture</t>
-        </is>
-      </c>
-      <c r="D37" s="15" t="inlineStr">
-        <is>
-          <t>Architecture</t>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>Logging / monitoring</t>
+          <t>Subscription webhooks</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Ensure logging/monitoring so failures are visible ('a lot of things have been downed').</t>
+          <t>Handle checkout.session.completed/subscription.created (provision + set first-period quota), invoice.paid (RESET monthly quota = new period), subscription.updated (status, cancel_at_period_end, plan change), subscription.deleted, invoice.payment_failed (past_due + restrict). Verify signatures, idempotent.</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>decision 13.06</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
@@ -2297,8 +2297,302 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Quota enforcement (use-it-or-lose-it)</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>On each ad-creative/ad-video generation: if period used_count &lt; limit -&gt; allow + increment atomically, else BLOCK with reset date. No rollover, no overage (block until next cycle).</t>
+        </is>
+      </c>
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>decision 13.06</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I38" s="6" t="inlineStr"/>
+      <c r="J38" s="6" t="inlineStr"/>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Plans UI + usage display</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>New Plans/Subscription section (tier cards), Subscribe CTA. Current plan with remaining-this-month (e.g. 'Creatives 3/5, Videos 2/3'), renews date, Manage/Cancel -&gt; Customer Portal. Disable generate + show reset date when exhausted; past_due banner.</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>decision 13.06</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr"/>
+      <c r="J39" s="6" t="inlineStr"/>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade/downgrade handling</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>Mid-cycle plan change: Stripe handles billing proration; quota change applies from next period (v1). Refine later.</t>
+        </is>
+      </c>
+      <c r="G40" s="9" t="inlineStr">
+        <is>
+          <t>decision 13.06</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>later</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr"/>
+      <c r="J40" s="6" t="inlineStr"/>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>ARCH1</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Multi-tenancy / org_id from day 1</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>Introduce org_id / tenant_id in the data model, auth &amp; storage now (even if full white-label comes later). Retrofitting is expensive.</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>handoff</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr"/>
+      <c r="J41" s="6" t="inlineStr"/>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>ARCH2</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Async jobs / queue</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>Run AI generation &amp; video rendering via a queue + status + webhooks; never synchronously inside the request.</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>handoff</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I42" s="6" t="inlineStr"/>
+      <c r="J42" s="6" t="inlineStr"/>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>ARCH3</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Logging / monitoring</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>Ensure logging/monitoring so failures are visible ('a lot of things have been downed').</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr"/>
+      <c r="J43" s="6" t="inlineStr"/>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:K37"/>
+  <autoFilter ref="A3:K43"/>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>

</xml_diff>